<commit_message>
docs: slowniczek - odpowiedzi na pytania do tlumaczy (pt obreia de Natal, es el senor, it pane dolce nuziale, de langer Bauernrock, cs wolacz Marysio)
</commit_message>
<xml_diff>
--- a/tools/Translations/slowniczek.xlsx
+++ b/tools/Translations/slowniczek.xlsx
@@ -2264,7 +2264,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Właściciel majątku i wsi (szlachcic z dworu); w tekście nie pojawia się osobiście. Prolog: oddaje pustki pod karczunek za niski czynsz; r4: sprzedał Urbaniakowi wyrąb; r11: „Jaśnie pan dziedzic zarządza obławę”, płaci za skórę wilka. „Jaśnie pan” = uniżona formuła chłopa lub sługi: en „His Lordship the squire”, de „der gnädige Herr”, cs/sk „milostpán”, ja 地主様. „Dwór” (strzelcy z dworu, dworska stodoła): en the manor, de der Gutshof, cs panský dvůr, sk kaštieľ. Bez współczesnych słów typu „właściciel ziemski”.</t>
+          <t xml:space="preserve">Właściciel majątku i wsi (szlachcic z dworu); w tekście nie pojawia się osobiście. Prolog: oddaje pustki pod karczunek za niski czynsz; r4: sprzedał Urbaniakowi wyrąb; r11: „Jaśnie pan dziedzic zarządza obławę”, płaci za skórę wilka. „Jaśnie pan” = uniżona formuła chłopa lub sługi: en „His Lordship the squire”, de „der gnädige Herr”, cs/sk „milostpán”, ja 地主様. „Dwór” (strzelcy z dworu, dworska stodoła): en the manor, de der Gutshof, cs panský dvůr, sk kaštieľ. Bez współczesnych słów typu „właściciel ziemski”. es: „el señor” w ustach postaci i w zwrotach, w narracji „el señor de la finca”; „terrateniente” tylko tam, gdzie narrator opisuje stosunki własnościowe (termin opisowy, z odcieniem krytycznym); „hacendado” brzmi latynoamerykańsko.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">el terrateniente</t>
+          <t xml:space="preserve">el señor</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kożuch: okrycie z owczej skóry, wełną do środka. Motyw „kożuch wywrócony włosiem na wierzch” (starzec / Pan Lasu r2, r9, r16, r20; Jaromir r3) oddać dosłownie: en „a sheepskin turned fleece-out”, de „mit dem Fell nach außen”, cs „kožich obrácený srstí ven”, sk „kožuch obrátený srsťou von”. Kapota: sukienne okrycie wierzchnie z podszewką (r9 kapota Franka „podszewką na wierzch”, r16 i r18 Jaromira „szwami na wierzch”) — zwykły wyraz na płaszcz lub kurtkę, bez egzotyzmu. To dwie różne rzeczy, nie mieszać. Sukmana (prolog, r3) — tak samo zwykły wyraz na chłopskie okrycie z grubego sukna. Uwaga: „tęczowy kożuch” na wodzie (r16) to warstwa na powierzchni (en film, de Schicht, cs povlak), nie ubranie.</t>
+          <t xml:space="preserve">Kożuch: okrycie z owczej skóry, wełną do środka. Motyw „kożuch wywrócony włosiem na wierzch” (starzec / Pan Lasu r2, r9, r16, r20; Jaromir r3) oddać dosłownie: en „a sheepskin turned fleece-out”, de „mit dem Fell nach außen”, cs „kožich obrácený srstí ven”, sk „kožuch obrátený srsťou von”. Kapota: sukienne okrycie wierzchnie z podszewką (r9 kapota Franka „podszewką na wierzch”, r16 i r18 Jaromira „szwami na wierzch”) — zwykły wyraz na płaszcz lub kurtkę, bez egzotyzmu. To dwie różne rzeczy, nie mieszać. Sukmana (prolog, r3) — tak samo zwykły wyraz na chłopskie okrycie z grubego sukna. Uwaga: „tęczowy kożuch” na wodzie (r16) to warstwa na powierzchni (en film, de Schicht, cs povlak), nie ubranie. de: kapota to długie okrycie — „langer Bauernrock” / „langer Rock”, nie „Joppe” (krótka kurtka bawarska).</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Schafspelz / Joppe</t>
+          <t xml:space="preserve">Schafspelz / langer Bauernrock</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -6016,7 +6016,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cienki biały wafel łamany w Wigilię; kładziony na talerzu dla wędrowca. W tekście też porównanie „cienki jak opłatek” (lód) — oddać naturalnym porównaniem (en „wafer-thin”, de „hauchdünn wie eine Oblate”).</t>
+          <t xml:space="preserve">Cienki biały wafel łamany w Wigilię; kładziony na talerzu dla wędrowca. W tekście też porównanie „cienki jak opłatek” (lód) — oddać naturalnym porównaniem (en „wafer-thin”, de „hauchdünn wie eine Oblate”). pt: „obreia” (niekonsekrowany wafel), nie „hóstia” (Eucharystia); przy pierwszym wystąpieniu można „opłatek (obreia de Natal)”, dalej „obreia”. Wariant docelowy: brazylijski.</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hóstia de Natal</t>
+          <t xml:space="preserve">obreia de Natal</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -6418,7 +6418,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weselny placek drożdżowy (Hanka piecze je z miodem); poczęstunek dla starca w noc oczepin.</t>
+          <t xml:space="preserve">Weselny placek drożdżowy, słodki (Hanka piecze je z miodem); poczęstunek dla starca w noc oczepin. it: nie „focaccia” (płaski wytrawny chleb) ani „torta nuziale” (nowoczesny tort); przy pierwszym wystąpieniu można „kołacz, il pane nuziale”.</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">focaccia nuziale</t>
+          <t xml:space="preserve">pane dolce nuziale</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr">
@@ -8664,77 +8664,77 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Otwarte pytania do natywnych tłumaczy</t>
+          <t xml:space="preserve">Rozstrzygnięte przez autora</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. cs: wołacz „Marysio!” (przyjęty) czy „Marysie!”?</t>
+          <t xml:space="preserve">• en „Mr Ignacy” (nie „Master”).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. pt: „hóstia de Natal” kojarzy się z hostią konsekrowaną — czy jest lepsze słowo na opłatek?</t>
+          <t xml:space="preserve">• cs/sk „Staš” zamiast „Staś”.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. es „terrateniente” (dziedzic), it „focaccia nuziale” (kołacz), de „Joppe” (kapota) — potwierdzić.</t>
+          <t xml:space="preserve">• cs topielec = „utopec”.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• es kapliczka = „humilladero”.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rozstrzygnięte przez autora</t>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• sk „podhodenec” zostaje: podrzutek, dziecko podrzucone komuś, coś podrzuconego, obcego.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• en „Mr Ignacy” (nie „Master”).</t>
+          <t xml:space="preserve">• cs wołacz „Marysio!” — polskie imię na -a odmienia się jak czeskie żeńskie (Jana → Jano, Maria → Mario); „Marysie!” tylko przy sczeszczonym mianowniku, czego nie chcemy.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• cs/sk „Staš” zamiast „Staś”.</t>
+          <t xml:space="preserve">• pt opłatek = „obreia de Natal” (nie „hóstia”, kojarzy się z Eucharystią).</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• cs topielec = „utopec”.</t>
+          <t xml:space="preserve">• es dziedzic = „el señor” (w narracji „el señor de la finca”), nie „terrateniente”.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• es kapliczka = „humilladero”.</t>
+          <t xml:space="preserve">• it kołacz = „pane dolce nuziale” (nie „focaccia”, nie „torta nuziale”).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• sk „podhodenec” zostaje: podrzutek, dziecko podrzucone komuś, coś podrzuconego, obcego.</t>
+          <t xml:space="preserve">• de kapota = „langer Bauernrock” (nie „Joppe” — to krótka kurtka).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: slowniczek - oplatek it 'la cialda di Natale', fr polskie 'l'oplatek' z objasnieniem
</commit_message>
<xml_diff>
--- a/tools/Translations/slowniczek.xlsx
+++ b/tools/Translations/slowniczek.xlsx
@@ -6016,7 +6016,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cienki biały wafel łamany w Wigilię; kładziony na talerzu dla wędrowca. W tekście też porównanie „cienki jak opłatek” (lód) — oddać naturalnym porównaniem (en „wafer-thin”, de „hauchdünn wie eine Oblate”). pt: „obreia” (niekonsekrowany wafel), nie „hóstia” (Eucharystia); przy pierwszym wystąpieniu można „opłatek (obreia de Natal)”, dalej „obreia”. Wariant docelowy: brazylijski.</t>
+          <t xml:space="preserve">Cienki biały wafel łamany w Wigilię; kładziony na talerzu dla wędrowca. W tekście też porównanie „cienki jak opłatek” (lód) — oddać naturalnym porównaniem (en „wafer-thin”, de „hauchdünn wie eine Oblate”). pt: „obreia” (niekonsekrowany wafel), nie „hóstia” (Eucharystia); przy pierwszym wystąpieniu można „opłatek (obreia de Natal)”, dalej „obreia”. Wariant docelowy: brazylijski. it: „cialda” (neutralny wafel; „ostia” i „oblata” kojarzą się z liturgią), porównanie „sottile come una cialda”. fr: polskie słowo „l’opłatek” (jedyny przedmiot, który zostaje po polsku — „hostie” = Eucharystia, „oublie” = dziś słodki rożek); przy pierwszym wystąpieniu „l’opłatek, la fine galette de pain azyme qu’on rompt à la veille de Noël”, porównanie z lodem „mince comme une feuille”.</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -6041,12 +6041,12 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">l’hostie de Noël</t>
+          <t xml:space="preserve">l’opłatek</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">l’ostia di Natale</t>
+          <t xml:space="preserve">la cialda di Natale</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -8720,33 +8720,40 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• es dziedzic = „el señor” (w narracji „el señor de la finca”), nie „terrateniente”.</t>
+          <t xml:space="preserve">• it opłatek = „la cialda di Natale”; fr opłatek = polskie „l’opłatek” z objaśnieniem przy pierwszym wystąpieniu (jedyny przedmiot, który zostaje po polsku).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• it kołacz = „pane dolce nuziale” (nie „focaccia”, nie „torta nuziale”).</t>
+          <t xml:space="preserve">• es dziedzic = „el señor” (w narracji „el señor de la finca”), nie „terrateniente”.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• de kapota = „langer Bauernrock” (nie „Joppe” — to krótka kurtka).</t>
+          <t xml:space="preserve">• it kołacz = „pane dolce nuziale” (nie „focaccia”, nie „torta nuziale”).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Dopisane hasła: Borowy, świta, gajowy, opłatek, kołacz, błędne ognie, dziedzic, kożuch/kapota, drużba, ruble srebrem (szarwark pominięty — nie pada w tekście gry).</t>
+          <t xml:space="preserve">• de kapota = „langer Bauernrock” (nie „Joppe” — to krótka kurtka).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Dopisane hasła: Borowy, świta, gajowy, opłatek, kołacz, błędne ognie, dziedzic, kożuch/kapota, drużba, ruble srebrem (szarwark pominięty — nie pada w tekście gry).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">• cs/sk: Marysia i Jadwisia odmieniane jak imiona na -ia, dzierżawczość dopełniaczem („dřeváky Marysie”).</t>
         </is>

</xml_diff>